<commit_message>
more figure and source data formatting
</commit_message>
<xml_diff>
--- a/sourcedatadir/Source_Data_Fig3.xlsx
+++ b/sourcedatadir/Source_Data_Fig3.xlsx
@@ -11,12 +11,13 @@
     <sheet name="3D_heatmap_types_env" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="3E_k_type_novel_old" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="3F_Ktype_novel_unknown" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="3E_k_type_novel_old_environment" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
   <si>
     <t xml:space="preserve">total</t>
   </si>
@@ -385,6 +386,9 @@
   <si>
     <t xml:space="preserve">normcount</t>
   </si>
+  <si>
+    <t xml:space="preserve">uncharacterised</t>
+  </si>
 </sst>
 </file>
 
@@ -18211,7 +18215,7 @@
         <v>28</v>
       </c>
       <c r="B32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C32" t="n">
         <v>55</v>
@@ -18225,7 +18229,7 @@
         <v>29</v>
       </c>
       <c r="B33" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C33" t="n">
         <v>49</v>
@@ -18239,7 +18243,7 @@
         <v>30</v>
       </c>
       <c r="B34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C34" t="n">
         <v>19</v>
@@ -18253,7 +18257,7 @@
         <v>31</v>
       </c>
       <c r="B35" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C35" t="n">
         <v>68</v>
@@ -18267,7 +18271,7 @@
         <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C36" t="n">
         <v>35</v>
@@ -18281,7 +18285,7 @@
         <v>33</v>
       </c>
       <c r="B37" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C37" t="n">
         <v>24</v>
@@ -18295,7 +18299,7 @@
         <v>35</v>
       </c>
       <c r="B38" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C38" t="n">
         <v>57</v>
@@ -18309,7 +18313,7 @@
         <v>36</v>
       </c>
       <c r="B39" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C39" t="n">
         <v>56</v>
@@ -18323,7 +18327,7 @@
         <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C40" t="n">
         <v>45</v>
@@ -18337,7 +18341,7 @@
         <v>38</v>
       </c>
       <c r="B41" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C41" t="n">
         <v>70</v>
@@ -18351,7 +18355,7 @@
         <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C42" t="n">
         <v>27</v>
@@ -18365,7 +18369,7 @@
         <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C43" t="n">
         <v>21</v>
@@ -18379,7 +18383,7 @@
         <v>41</v>
       </c>
       <c r="B44" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C44" t="n">
         <v>38</v>
@@ -18393,7 +18397,7 @@
         <v>42</v>
       </c>
       <c r="B45" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C45" t="n">
         <v>24</v>
@@ -18407,7 +18411,7 @@
         <v>43</v>
       </c>
       <c r="B46" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C46" t="n">
         <v>31</v>
@@ -18421,7 +18425,7 @@
         <v>44</v>
       </c>
       <c r="B47" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C47" t="n">
         <v>28</v>
@@ -18435,7 +18439,7 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C48" t="n">
         <v>21</v>
@@ -18449,7 +18453,7 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C49" t="n">
         <v>17</v>
@@ -18463,7 +18467,7 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C50" t="n">
         <v>20</v>
@@ -18477,7 +18481,7 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C51" t="n">
         <v>28</v>
@@ -18491,7 +18495,7 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C52" t="n">
         <v>7</v>
@@ -18505,7 +18509,7 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C53" t="n">
         <v>17</v>
@@ -18519,7 +18523,7 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C54" t="n">
         <v>18</v>
@@ -18533,7 +18537,7 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C55" t="n">
         <v>12</v>
@@ -18547,7 +18551,7 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C56" t="n">
         <v>25</v>
@@ -18561,7 +18565,7 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C57" t="n">
         <v>5</v>
@@ -18575,7 +18579,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C58" t="n">
         <v>6</v>
@@ -18589,7 +18593,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C59" t="n">
         <v>12</v>
@@ -18603,7 +18607,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C60" t="n">
         <v>6</v>
@@ -18617,7 +18621,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C61" t="n">
         <v>8</v>
@@ -18631,7 +18635,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C62" t="n">
         <v>5</v>
@@ -18645,7 +18649,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C63" t="n">
         <v>8</v>
@@ -18659,7 +18663,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C64" t="n">
         <v>10</v>
@@ -18673,7 +18677,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C65" t="n">
         <v>10</v>
@@ -18687,7 +18691,7 @@
         <v>66</v>
       </c>
       <c r="B66" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C66" t="n">
         <v>3</v>
@@ -18701,7 +18705,7 @@
         <v>67</v>
       </c>
       <c r="B67" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C67" t="n">
         <v>3</v>
@@ -18715,7 +18719,7 @@
         <v>68</v>
       </c>
       <c r="B68" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C68" t="n">
         <v>1</v>
@@ -18729,7 +18733,7 @@
         <v>69</v>
       </c>
       <c r="B69" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C69" t="n">
         <v>1</v>
@@ -18743,7 +18747,7 @@
         <v>70</v>
       </c>
       <c r="B70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C70" t="n">
         <v>1</v>
@@ -18757,7 +18761,7 @@
         <v>71</v>
       </c>
       <c r="B71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C71" t="n">
         <v>2</v>
@@ -18771,7 +18775,7 @@
         <v>72</v>
       </c>
       <c r="B72" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C72" t="n">
         <v>1</v>
@@ -18785,7 +18789,7 @@
         <v>73</v>
       </c>
       <c r="B73" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C73" t="n">
         <v>5</v>
@@ -18799,7 +18803,7 @@
         <v>74</v>
       </c>
       <c r="B74" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C74" t="n">
         <v>1</v>
@@ -18813,7 +18817,7 @@
         <v>75</v>
       </c>
       <c r="B75" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C75" t="n">
         <v>32</v>
@@ -18827,7 +18831,7 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C76" t="n">
         <v>2</v>
@@ -18841,7 +18845,7 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C77" t="n">
         <v>1</v>
@@ -18855,7 +18859,7 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C78" t="n">
         <v>1</v>
@@ -18869,7 +18873,7 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C79" t="n">
         <v>1</v>
@@ -18883,7 +18887,7 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C80" t="n">
         <v>1</v>
@@ -18897,7 +18901,7 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C81" t="n">
         <v>3</v>
@@ -18911,7 +18915,7 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C82" t="n">
         <v>1</v>
@@ -18925,7 +18929,7 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C83" t="n">
         <v>1</v>
@@ -18939,13 +18943,415 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C84" t="n">
         <v>1</v>
       </c>
       <c r="D84" t="n">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>66.6666666666667</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" t="n">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E3" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="n">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" t="n">
+        <v>83.3333333333333</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" t="n">
+        <v>142</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="n">
+        <v>65</v>
+      </c>
+      <c r="E5" t="n">
+        <v>45.7746478873239</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" t="n">
+        <v>171</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="n">
+        <v>111</v>
+      </c>
+      <c r="E6" t="n">
+        <v>64.9122807017544</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" t="n">
+        <v>181</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" t="n">
+        <v>146</v>
+      </c>
+      <c r="E7" t="n">
+        <v>80.6629834254144</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" t="n">
+        <v>227</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="n">
+        <v>181</v>
+      </c>
+      <c r="E8" t="n">
+        <v>79.7356828193833</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" t="n">
+        <v>287</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="n">
+        <v>157</v>
+      </c>
+      <c r="E9" t="n">
+        <v>54.7038327526132</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" t="n">
+        <v>404</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="n">
+        <v>268</v>
+      </c>
+      <c r="E10" t="n">
+        <v>66.3366336633663</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" t="n">
+        <v>432</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" t="n">
+        <v>302</v>
+      </c>
+      <c r="E11" t="n">
+        <v>69.9074074074074</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4321</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3541</v>
+      </c>
+      <c r="E12" t="n">
+        <v>81.9486230039343</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>33.3333333333333</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" t="n">
+        <v>24</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>122</v>
+      </c>
+      <c r="B15" t="n">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" t="n">
+        <v>16.6666666666667</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>122</v>
+      </c>
+      <c r="B16" t="n">
+        <v>142</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="n">
+        <v>77</v>
+      </c>
+      <c r="E16" t="n">
+        <v>54.2253521126761</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B17" t="n">
+        <v>171</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="n">
+        <v>60</v>
+      </c>
+      <c r="E17" t="n">
+        <v>35.0877192982456</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>122</v>
+      </c>
+      <c r="B18" t="n">
+        <v>181</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" t="n">
+        <v>35</v>
+      </c>
+      <c r="E18" t="n">
+        <v>19.3370165745856</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B19" t="n">
+        <v>227</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="n">
+        <v>46</v>
+      </c>
+      <c r="E19" t="n">
+        <v>20.2643171806167</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" t="n">
+        <v>287</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="n">
+        <v>130</v>
+      </c>
+      <c r="E20" t="n">
+        <v>45.2961672473868</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" t="n">
+        <v>404</v>
+      </c>
+      <c r="C21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" t="n">
+        <v>136</v>
+      </c>
+      <c r="E21" t="n">
+        <v>33.6633663366337</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>122</v>
+      </c>
+      <c r="B22" t="n">
+        <v>432</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" t="n">
+        <v>130</v>
+      </c>
+      <c r="E22" t="n">
+        <v>30.0925925925926</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4321</v>
+      </c>
+      <c r="C23" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" t="n">
+        <v>780</v>
+      </c>
+      <c r="E23" t="n">
+        <v>18.0513769960657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>